<commit_message>
NTGNT.CO CR:c|low|missing. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/NTGNT.CO.xlsx
+++ b/data/cox_xlsx/NTGNT.CO.xlsx
@@ -3424,21 +3424,11 @@
       <c r="I43" s="15"/>
       <c r="J43" s="15"/>
       <c r="K43" s="15"/>
-      <c r="L43" s="17">
-        <v>3.39</v>
-      </c>
-      <c r="M43" s="17">
-        <v>3.55</v>
-      </c>
-      <c r="N43" s="17">
-        <v>15.29</v>
-      </c>
-      <c r="O43" s="17">
-        <v>9.91</v>
-      </c>
-      <c r="P43" s="17">
-        <v>13.22</v>
-      </c>
+      <c r="L43" s="17"/>
+      <c r="M43" s="17"/>
+      <c r="N43" s="17"/>
+      <c r="O43" s="17"/>
+      <c r="P43" s="17"/>
       <c r="Q43" s="15"/>
       <c r="R43" s="15"/>
       <c r="S43" s="15"/>

</xml_diff>